<commit_message>
Updated rule to workaround issue #873
</commit_message>
<xml_diff>
--- a/rules/CORE-000598/negative/01/data/unit-test-coreid-CG0413-negative.xlsx
+++ b/rules/CORE-000598/negative/01/data/unit-test-coreid-CG0413-negative.xlsx
@@ -3,8 +3,10 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Datasets" sheetId="1" r:id="rId1"/>
-    <sheet name="alb.xpt" sheetId="2" r:id="rId2"/>
+    <sheet name="Library" sheetId="1" r:id="rId1"/>
+    <sheet name="Datasets" sheetId="2" r:id="rId2"/>
+    <sheet name="Validation" sheetId="3" r:id="rId3"/>
+    <sheet name="alb.xpt" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -34,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -55,14 +57,10 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
       <i/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -75,13 +73,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor rgb="00FFFFCC"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -105,14 +97,13 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -448,18 +439,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
-        <v>Filename</v>
+        <v>Product</v>
       </c>
       <c r="B1" s="3" t="str">
-        <v>Label</v>
+        <v>Version</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="str">
-        <v>alb.xpt</v>
+        <v>sdtmig</v>
       </c>
       <c r="B2" s="4" t="str">
-        <v>Laboratory Test Results A</v>
+        <v>3-4</v>
       </c>
     </row>
   </sheetData>
@@ -471,28 +462,86 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:B2"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="str">
+      <c r="A1" s="3" t="str">
+        <v>Filename</v>
+      </c>
+      <c r="B1" s="3" t="str">
+        <v>Label</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="str">
+        <v>alb.xpt</v>
+      </c>
+      <c r="B2" s="4" t="str">
+        <v>Laboratory Test Results A</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="str">
+        <v>Error group</v>
+      </c>
+      <c r="B1" s="3" t="str">
+        <v>Sheet</v>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v>Error level</v>
+      </c>
+      <c r="D1" s="3" t="str">
+        <v>Row num</v>
+      </c>
+      <c r="E1" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="F1" s="3" t="str">
+        <v>Error value</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="str">
         <v>STUDYID</v>
       </c>
-      <c r="B1" s="5" t="str">
+      <c r="B1" s="3" t="str">
         <v>DOMAIN</v>
       </c>
-      <c r="C1" s="5" t="str">
+      <c r="C1" s="3" t="str">
         <v>USUBJID</v>
       </c>
-      <c r="D1" s="5" t="str">
+      <c r="D1" s="3" t="str">
         <v>LBTESTCD</v>
       </c>
-      <c r="E1" s="5" t="str">
+      <c r="E1" s="3" t="str">
         <v>LBTEST</v>
       </c>
-      <c r="F1" s="5" t="str">
+      <c r="F1" s="3" t="str">
         <v>LBSTREFC</v>
       </c>
-      <c r="G1" s="5" t="str">
+      <c r="G1" s="3" t="str">
         <v>LBSTREFN</v>
       </c>
     </row>
@@ -506,10 +555,10 @@
       <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="5" t="str">
         <v>Lab Test or Examination Short Name</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="5" t="str">
         <v>Lab Test or Examination Name</v>
       </c>
       <c r="F2" s="5" t="str">
@@ -529,10 +578,10 @@
       <c r="C3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="D3" s="6" t="str">
+      <c r="D3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="E3" s="6" t="str">
+      <c r="E3" s="5" t="str">
         <v>Char</v>
       </c>
       <c r="F3" s="5" t="str">
@@ -552,10 +601,10 @@
       <c r="C4" s="5">
         <v>8</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <v>50</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <v>50</v>
       </c>
       <c r="F4" s="5">
@@ -566,31 +615,54 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="str">
+      <c r="A5" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="5" t="str">
+      <c r="B5" s="4" t="str">
         <v>LB</v>
       </c>
-      <c r="C5" s="5" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="5" t="str">
-        <v/>
-      </c>
-      <c r="E5" s="5" t="str">
-        <v/>
-      </c>
-      <c r="F5" s="5" t="str">
+      <c r="D5" s="4" t="str">
+        <v>TEST</v>
+      </c>
+      <c r="E5" s="4" t="str">
+        <v>Test</v>
+      </c>
+      <c r="F5" s="4" t="str">
         <v>ABC</v>
       </c>
-      <c r="G5" s="5" t="str">
+      <c r="G5" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B6" s="4" t="str">
+        <v>LB</v>
+      </c>
+      <c r="C6" s="4" t="str">
+        <v>CDISC001</v>
+      </c>
+      <c r="D6" s="4" t="str">
+        <v>TEST</v>
+      </c>
+      <c r="E6" s="4" t="str">
+        <v>Test</v>
+      </c>
+      <c r="F6" s="4" t="str">
+        <v>ABC</v>
+      </c>
+      <c r="G6" s="4" t="str">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added rows to the Validation sheet for negative test data
</commit_message>
<xml_diff>
--- a/rules/CORE-000598/negative/01/data/unit-test-coreid-CG0413-negative.xlsx
+++ b/rules/CORE-000598/negative/01/data/unit-test-coreid-CG0413-negative.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -59,8 +59,13 @@
       <name val="Calibri"/>
       <i/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -68,6 +73,12 @@
     </fill>
     <fill>
       <patternFill patternType="gray125">
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFCC"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -97,13 +108,14 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -489,7 +501,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -511,9 +523,69 @@
         <v>Error value</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="str">
+        <v>alb.xpt</v>
+      </c>
+      <c r="C2" s="4" t="str">
+        <v>Dataset</v>
+      </c>
+      <c r="D2" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E2" s="4" t="str">
+        <v>dataset_name</v>
+      </c>
+      <c r="F2" s="4" t="str">
+        <v>ALB</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>alb.xpt</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>Dataset</v>
+      </c>
+      <c r="D3" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E3" s="2" t="str">
+        <v>variable_name</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <v>DOMAIN</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>alb.xpt</v>
+      </c>
+      <c r="C4" s="2" t="str">
+        <v>Dataset</v>
+      </c>
+      <c r="D4" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E4" s="2" t="str">
+        <v>variable_value</v>
+      </c>
+      <c r="F4" s="2" t="str">
+        <v>LB</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -558,59 +630,59 @@
       <c r="D2" s="5" t="str">
         <v>Lab Test or Examination Short Name</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Lab Test or Examination Name</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Character Reference Result</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Numeric Reference Result in Std Units</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
+      <c r="A3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="B3" s="5" t="str">
+      <c r="B3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="C3" s="5" t="str">
+      <c r="C3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="D3" s="5" t="str">
+      <c r="D3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="E3" s="5" t="str">
+      <c r="E3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="F3" s="5" t="str">
+      <c r="F3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="G3" s="5" t="str">
+      <c r="G3" s="6" t="str">
         <v>Num</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>12</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="6">
         <v>8</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="6">
         <v>50</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="6">
         <v>50</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="6">
         <v>8</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="6">
         <v>8</v>
       </c>
     </row>

</xml_diff>